<commit_message>
Applied first css for apacy svg handling implementest  and applied  function forremoval of texttype
</commit_message>
<xml_diff>
--- a/Lingvistik_proj/ausen-emma_head_lingvistik.xlsx
+++ b/Lingvistik_proj/ausen-emma_head_lingvistik.xlsx
@@ -543,7 +543,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ausen-emma_S_2341_L_1</t>
+          <t>ausen-emma_S#2341_L#1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ausen-emma_S_2727_L_2</t>
+          <t>ausen-emma_S#2727_L#2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -703,7 +703,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ausen-emma_S_2936_L_3</t>
+          <t>ausen-emma_S#2936_L#3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -779,7 +779,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ausen-emma_S_11884_L_4</t>
+          <t>ausen-emma_S#11884_L#4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -859,7 +859,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ausen-emma_S_13694_L_5</t>
+          <t>ausen-emma_S#13694_L#5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -939,7 +939,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ausen-emma_S_16168_L_6</t>
+          <t>ausen-emma_S#16168_L#6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1019,7 +1019,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ausen-emma_S_24059_L_7</t>
+          <t>ausen-emma_S#24059_L#7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1099,7 +1099,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ausen-emma_S_26305_L_8</t>
+          <t>ausen-emma_S#26305_L#8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ausen-emma_S_35885_L_9</t>
+          <t>ausen-emma_S#35885_L#9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1267,7 +1267,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ausen-emma_S_39630_L_10</t>
+          <t>ausen-emma_S#39630_L#10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1351,7 +1351,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ausen-emma_S_40374_L_11</t>
+          <t>ausen-emma_S#40374_L#11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ausen-emma_S_41464_L_12</t>
+          <t>ausen-emma_S#41464_L#12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1511,7 +1511,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ausen-emma_S_52610_L_13</t>
+          <t>ausen-emma_S#52610_L#13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1595,7 +1595,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ausen-emma_S_68950_L_14</t>
+          <t>ausen-emma_S#68950_L#14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1679,7 +1679,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ausen-emma_S_76580_L_15</t>
+          <t>ausen-emma_S#76580_L#15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1751,7 +1751,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ausen-emma_S_83449_L_16</t>
+          <t>ausen-emma_S#83449_L#16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1831,7 +1831,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ausen-emma_S_86346_L_17</t>
+          <t>ausen-emma_S#86346_L#17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1915,7 +1915,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ausen-emma_S_86843_L_18</t>
+          <t>ausen-emma_S#86843_L#18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1991,7 +1991,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ausen-emma_S_93472_L_19</t>
+          <t>ausen-emma_S#93472_L#19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2075,7 +2075,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ausen-emma_S_94613_L_20</t>
+          <t>ausen-emma_S#94613_L#20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2159,7 +2159,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ausen-emma_S_100395_L_21</t>
+          <t>ausen-emma_S#100395_L#21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2239,7 +2239,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ausen-emma_S_102584_L_22</t>
+          <t>ausen-emma_S#102584_L#22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2323,7 +2323,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ausen-emma_S_104031_L_23</t>
+          <t>ausen-emma_S#104031_L#23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2403,7 +2403,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ausen-emma_S_104106_L_24</t>
+          <t>ausen-emma_S#104106_L#24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2487,7 +2487,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ausen-emma_S_107310_L_25</t>
+          <t>ausen-emma_S#107310_L#25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ausen-emma_S_112173_L_26</t>
+          <t>ausen-emma_S#112173_L#26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2647,7 +2647,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ausen-emma_S_116281_L_27</t>
+          <t>ausen-emma_S#116281_L#27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2727,7 +2727,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ausen-emma_S_119658_L_28</t>
+          <t>ausen-emma_S#119658_L#28</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2811,7 +2811,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ausen-emma_S_126934_L_29</t>
+          <t>ausen-emma_S#126934_L#29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2895,7 +2895,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ausen-emma_S_128454_L_30</t>
+          <t>ausen-emma_S#128454_L#30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2975,7 +2975,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ausen-emma_S_129603_L_31</t>
+          <t>ausen-emma_S#129603_L#31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3059,7 +3059,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ausen-emma_S_136556_L_32</t>
+          <t>ausen-emma_S#136556_L#32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3139,7 +3139,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ausen-emma_S_149874_L_33</t>
+          <t>ausen-emma_S#149874_L#33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3223,7 +3223,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ausen-emma_S_150755_L_34</t>
+          <t>ausen-emma_S#150755_L#34</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3307,7 +3307,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ausen-emma_S_151760_L_35</t>
+          <t>ausen-emma_S#151760_L#35</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3391,7 +3391,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ausen-emma_S_156585_L_36</t>
+          <t>ausen-emma_S#156585_L#36</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3475,7 +3475,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ausen-emma_S_161276_L_37</t>
+          <t>ausen-emma_S#161276_L#37</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3551,7 +3551,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ausen-emma_S_174778_L_38</t>
+          <t>ausen-emma_S#174778_L#38</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3635,7 +3635,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ausen-emma_S_178199_L_39</t>
+          <t>ausen-emma_S#178199_L#39</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3715,7 +3715,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ausen-emma_S_186688_L_40</t>
+          <t>ausen-emma_S#186688_L#40</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3787,7 +3787,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ausen-emma_S_188417_L_41</t>
+          <t>ausen-emma_S#188417_L#41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3867,7 +3867,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ausen-emma_S_188454_L_42</t>
+          <t>ausen-emma_S#188454_L#42</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">

</xml_diff>